<commit_message>
create images for bohrungen
</commit_message>
<xml_diff>
--- a/Boden/Torfzersetzung.xlsx
+++ b/Boden/Torfzersetzung.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nele\OneDrive - Technische Universität Ilmenau\Dokumente\Moore-Lichtenau-Meusebach\Boden\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D5D3C79-66FF-43F5-A636-E732E174484F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79BF8CEF-4F78-4744-9B63-8BAD40F96D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1DA430AB-B013-423E-A66C-CAABC9DD0E42}"/>
+    <workbookView xWindow="17595" yWindow="825" windowWidth="10980" windowHeight="13560" xr2:uid="{1DA430AB-B013-423E-A66C-CAABC9DD0E42}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -51,18 +51,6 @@
     <t>hum_num</t>
   </si>
   <si>
-    <t>Bor2</t>
-  </si>
-  <si>
-    <t>MT Nord</t>
-  </si>
-  <si>
-    <t>Bor4</t>
-  </si>
-  <si>
-    <t>MT Mitte</t>
-  </si>
-  <si>
     <t>2-1</t>
   </si>
   <si>
@@ -84,9 +72,6 @@
     <t>5-1</t>
   </si>
   <si>
-    <t>Bor6</t>
-  </si>
-  <si>
     <t>6-1</t>
   </si>
   <si>
@@ -96,18 +81,12 @@
     <t>6-2</t>
   </si>
   <si>
-    <t>MT Ost</t>
-  </si>
-  <si>
     <t>7-1</t>
   </si>
   <si>
     <t>7-2</t>
   </si>
   <si>
-    <t>Bor8</t>
-  </si>
-  <si>
     <t>8-1</t>
   </si>
   <si>
@@ -123,21 +102,9 @@
     <t>10-2</t>
   </si>
   <si>
-    <t>Bor11</t>
-  </si>
-  <si>
     <t>11-1</t>
   </si>
   <si>
-    <t>MN Mitte</t>
-  </si>
-  <si>
-    <t>Bor13</t>
-  </si>
-  <si>
-    <t>MN Ost</t>
-  </si>
-  <si>
     <t>12-1</t>
   </si>
   <si>
@@ -150,48 +117,27 @@
     <t>14-1</t>
   </si>
   <si>
-    <t>MN Süd</t>
-  </si>
-  <si>
     <t>15-1</t>
   </si>
   <si>
     <t>15-2</t>
   </si>
   <si>
-    <t>Bor16</t>
-  </si>
-  <si>
     <t>16-1</t>
   </si>
   <si>
-    <t>Bor17</t>
-  </si>
-  <si>
     <t>17-1</t>
   </si>
   <si>
-    <t>MN Nord</t>
-  </si>
-  <si>
     <t>18-1</t>
   </si>
   <si>
-    <t>Bor19</t>
-  </si>
-  <si>
     <t>19-1</t>
   </si>
   <si>
-    <t>Bor20</t>
-  </si>
-  <si>
     <t>20-1</t>
   </si>
   <si>
-    <t>Bor21</t>
-  </si>
-  <si>
     <t>21-1</t>
   </si>
   <si>
@@ -204,15 +150,9 @@
     <t>site</t>
   </si>
   <si>
-    <t>Bor23</t>
-  </si>
-  <si>
     <t>23-1</t>
   </si>
   <si>
-    <t>Bor24</t>
-  </si>
-  <si>
     <t>24-1</t>
   </si>
   <si>
@@ -222,72 +162,39 @@
     <t>24-3</t>
   </si>
   <si>
-    <t>Bor25</t>
-  </si>
-  <si>
     <t>25-1</t>
   </si>
   <si>
     <t>26-1</t>
   </si>
   <si>
-    <t>Bor27</t>
-  </si>
-  <si>
     <t>27-1</t>
   </si>
   <si>
-    <t>MT West</t>
-  </si>
-  <si>
     <t>28-1</t>
   </si>
   <si>
-    <t>Bor29</t>
-  </si>
-  <si>
     <t>29-1</t>
   </si>
   <si>
-    <t>Bor30</t>
-  </si>
-  <si>
     <t>30-1</t>
   </si>
   <si>
-    <t>Bor31</t>
-  </si>
-  <si>
     <t>31-1</t>
   </si>
   <si>
     <t>32-1</t>
   </si>
   <si>
-    <t>Bor33</t>
-  </si>
-  <si>
-    <t>Bor34</t>
-  </si>
-  <si>
     <t>34-1</t>
   </si>
   <si>
     <t>34-2</t>
   </si>
   <si>
-    <t>Bor35</t>
-  </si>
-  <si>
     <t>35-1</t>
   </si>
   <si>
-    <t>Bor36</t>
-  </si>
-  <si>
-    <t>Bor37</t>
-  </si>
-  <si>
     <t>25-2</t>
   </si>
   <si>
@@ -321,12 +228,6 @@
     <t>mt</t>
   </si>
   <si>
-    <t>Bor9</t>
-  </si>
-  <si>
-    <t>Bor10</t>
-  </si>
-  <si>
     <t>mn</t>
   </si>
   <si>
@@ -366,16 +267,115 @@
     <t>beide</t>
   </si>
   <si>
-    <t>MT süd</t>
-  </si>
-  <si>
-    <t>L Ost</t>
-  </si>
-  <si>
-    <t>L Mitte</t>
-  </si>
-  <si>
     <t>transekt nummer</t>
+  </si>
+  <si>
+    <t>Meusebach trocken West</t>
+  </si>
+  <si>
+    <t>Meusebach trocken Sued</t>
+  </si>
+  <si>
+    <t>Lichtenau Ost</t>
+  </si>
+  <si>
+    <t>BOR2</t>
+  </si>
+  <si>
+    <t>BOR4</t>
+  </si>
+  <si>
+    <t>BOR6</t>
+  </si>
+  <si>
+    <t>BOR8</t>
+  </si>
+  <si>
+    <t>BOR9</t>
+  </si>
+  <si>
+    <t>BOR10</t>
+  </si>
+  <si>
+    <t>BOR11</t>
+  </si>
+  <si>
+    <t>BOR13</t>
+  </si>
+  <si>
+    <t>BOR16</t>
+  </si>
+  <si>
+    <t>BOR17</t>
+  </si>
+  <si>
+    <t>BOR19</t>
+  </si>
+  <si>
+    <t>BOR20</t>
+  </si>
+  <si>
+    <t>BOR21</t>
+  </si>
+  <si>
+    <t>BOR23</t>
+  </si>
+  <si>
+    <t>BOR24</t>
+  </si>
+  <si>
+    <t>BOR25</t>
+  </si>
+  <si>
+    <t>BOR27</t>
+  </si>
+  <si>
+    <t>BOR29</t>
+  </si>
+  <si>
+    <t>BOR30</t>
+  </si>
+  <si>
+    <t>BOR31</t>
+  </si>
+  <si>
+    <t>BOR33</t>
+  </si>
+  <si>
+    <t>BOR34</t>
+  </si>
+  <si>
+    <t>BOR35</t>
+  </si>
+  <si>
+    <t>BOR36</t>
+  </si>
+  <si>
+    <t>BOR37</t>
+  </si>
+  <si>
+    <t>BOR3</t>
+  </si>
+  <si>
+    <t>BOR5</t>
+  </si>
+  <si>
+    <t>BOR7</t>
+  </si>
+  <si>
+    <t>BOR12</t>
+  </si>
+  <si>
+    <t>BOR14</t>
+  </si>
+  <si>
+    <t>BOR15</t>
+  </si>
+  <si>
+    <t>BOR18</t>
+  </si>
+  <si>
+    <t>BOR22</t>
   </si>
 </sst>
 </file>
@@ -737,6 +737,7 @@
   <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="32.85546875" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="3.85546875" customWidth="1"/>
   </cols>
@@ -764,21 +765,21 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="I1" t="s">
-        <v>107</v>
+        <v>74</v>
       </c>
       <c r="J1" t="s">
-        <v>115</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -791,24 +792,24 @@
         <v>88</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G2">
         <v>9</v>
       </c>
       <c r="H2" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I2" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>108</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -821,24 +822,24 @@
         <v>27</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G3">
         <v>8</v>
       </c>
       <c r="H3" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I3" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>108</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>27</v>
@@ -851,24 +852,24 @@
         <v>9</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G4">
         <v>9</v>
       </c>
       <c r="H4" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I4" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>84</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -881,18 +882,18 @@
         <v>40</v>
       </c>
       <c r="H5" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I5" t="s">
-        <v>110</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>109</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -905,24 +906,24 @@
         <v>100</v>
       </c>
       <c r="F6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G6">
         <v>9</v>
       </c>
       <c r="H6" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I6" t="s">
-        <v>111</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>85</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -935,24 +936,24 @@
         <v>40</v>
       </c>
       <c r="F7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G7">
         <v>9</v>
       </c>
       <c r="H7" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I7" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>85</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C8">
         <v>40</v>
@@ -965,24 +966,24 @@
         <v>60</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G8">
         <v>10</v>
       </c>
       <c r="H8" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I8" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>110</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -995,24 +996,24 @@
         <v>18</v>
       </c>
       <c r="F9" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G9">
         <v>9</v>
       </c>
       <c r="H9" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I9" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>110</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C10">
         <v>18</v>
@@ -1025,24 +1026,24 @@
         <v>45</v>
       </c>
       <c r="F10" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G10">
         <v>10</v>
       </c>
       <c r="H10" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I10" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1055,24 +1056,24 @@
         <v>50</v>
       </c>
       <c r="F11" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G11">
         <v>8</v>
       </c>
       <c r="H11" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I11" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C12">
         <v>50</v>
@@ -1085,24 +1086,24 @@
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G12">
         <v>10</v>
       </c>
       <c r="H12" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I12" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -1115,24 +1116,24 @@
         <v>92</v>
       </c>
       <c r="F13" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G13">
         <v>10</v>
       </c>
       <c r="H13" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I13" t="s">
-        <v>110</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1145,24 +1146,24 @@
         <v>15</v>
       </c>
       <c r="F14" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G14">
         <v>8</v>
       </c>
       <c r="H14" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I14" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C15">
         <v>15</v>
@@ -1175,24 +1176,24 @@
         <v>10</v>
       </c>
       <c r="F15" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G15">
         <v>10</v>
       </c>
       <c r="H15" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I15" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>89</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1205,24 +1206,24 @@
         <v>36</v>
       </c>
       <c r="F16" t="s">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="G16">
         <v>5</v>
       </c>
       <c r="H16" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I16" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>33</v>
+        <v>111</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -1235,24 +1236,24 @@
         <v>20</v>
       </c>
       <c r="F17" t="s">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="G17">
         <v>5</v>
       </c>
       <c r="H17" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I17" t="s">
-        <v>111</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>111</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="C18">
         <v>20</v>
@@ -1265,24 +1266,24 @@
         <v>19</v>
       </c>
       <c r="F18" t="s">
-        <v>102</v>
+        <v>69</v>
       </c>
       <c r="G18">
         <v>4</v>
       </c>
       <c r="H18" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I18" t="s">
-        <v>111</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -1295,24 +1296,24 @@
         <v>62</v>
       </c>
       <c r="F19" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="G19">
         <v>6</v>
       </c>
       <c r="H19" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I19" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>112</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -1325,24 +1326,24 @@
         <v>30</v>
       </c>
       <c r="F20" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G20">
         <v>9</v>
       </c>
       <c r="H20" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I20" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -1355,24 +1356,24 @@
         <v>20</v>
       </c>
       <c r="F21" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="G21">
         <v>1</v>
       </c>
       <c r="H21" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I21" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C22">
         <v>20</v>
@@ -1385,24 +1386,24 @@
         <v>16</v>
       </c>
       <c r="F22" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G22">
         <v>8</v>
       </c>
       <c r="H22" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I22" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -1415,24 +1416,24 @@
         <v>12</v>
       </c>
       <c r="F23" t="s">
-        <v>102</v>
+        <v>69</v>
       </c>
       <c r="G23">
         <v>4</v>
       </c>
       <c r="H23" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I23" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>45</v>
+        <v>92</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -1445,24 +1446,24 @@
         <v>28</v>
       </c>
       <c r="F24" t="s">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="G24">
         <v>5</v>
       </c>
       <c r="H24" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I24" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>47</v>
+        <v>114</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -1475,24 +1476,24 @@
         <v>55</v>
       </c>
       <c r="F25" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="G25">
         <v>6</v>
       </c>
       <c r="H25" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I25" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>49</v>
+        <v>93</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -1505,24 +1506,24 @@
         <v>55</v>
       </c>
       <c r="F26" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="G26">
         <v>6</v>
       </c>
       <c r="H26" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I26" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>51</v>
+        <v>94</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -1535,24 +1536,24 @@
         <v>100</v>
       </c>
       <c r="F27" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="G27">
         <v>6</v>
       </c>
       <c r="H27" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I27" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>53</v>
+        <v>95</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -1565,24 +1566,24 @@
         <v>5</v>
       </c>
       <c r="F28" t="s">
-        <v>102</v>
+        <v>69</v>
       </c>
       <c r="G28">
         <v>4</v>
       </c>
       <c r="H28" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I28" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>53</v>
+        <v>95</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="C29">
         <v>5</v>
@@ -1595,24 +1596,24 @@
         <v>69</v>
       </c>
       <c r="F29" t="s">
-        <v>105</v>
+        <v>72</v>
       </c>
       <c r="G29">
         <v>7</v>
       </c>
       <c r="H29" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I29" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -1625,24 +1626,24 @@
         <v>84</v>
       </c>
       <c r="F30" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G30">
         <v>8</v>
       </c>
       <c r="H30" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I30" t="s">
-        <v>111</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>58</v>
+        <v>96</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -1655,24 +1656,24 @@
         <v>100</v>
       </c>
       <c r="F31" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="G31">
         <v>6</v>
       </c>
       <c r="H31" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I31" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>60</v>
+        <v>97</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -1685,24 +1686,24 @@
         <v>35</v>
       </c>
       <c r="F32" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="G32">
         <v>1</v>
       </c>
       <c r="H32" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I32" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>60</v>
+        <v>97</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
       <c r="C33">
         <v>35</v>
@@ -1715,24 +1716,24 @@
         <v>5</v>
       </c>
       <c r="F33" t="s">
-        <v>106</v>
+        <v>73</v>
       </c>
       <c r="G33">
         <v>3</v>
       </c>
       <c r="H33" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I33" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>60</v>
+        <v>97</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="C34">
         <v>40</v>
@@ -1745,24 +1746,24 @@
         <v>60</v>
       </c>
       <c r="F34" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="G34">
         <v>6</v>
       </c>
       <c r="H34" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I34" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="C35">
         <v>0</v>
@@ -1775,24 +1776,24 @@
         <v>17</v>
       </c>
       <c r="F35" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="G35">
         <v>1</v>
       </c>
       <c r="H35" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I35" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="C36">
         <v>17</v>
@@ -1805,24 +1806,24 @@
         <v>7</v>
       </c>
       <c r="F36" t="s">
-        <v>102</v>
+        <v>69</v>
       </c>
       <c r="G36">
         <v>4</v>
       </c>
       <c r="H36" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I36" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="C37">
         <v>24</v>
@@ -1835,24 +1836,24 @@
         <v>28</v>
       </c>
       <c r="F37" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G37">
         <v>8</v>
       </c>
       <c r="H37" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I37" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>112</v>
+        <v>81</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -1865,24 +1866,24 @@
         <v>45</v>
       </c>
       <c r="F38" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G38">
         <v>8</v>
       </c>
       <c r="H38" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I38" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>67</v>
+        <v>99</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -1895,24 +1896,24 @@
         <v>35</v>
       </c>
       <c r="F39" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G39">
         <v>9</v>
       </c>
       <c r="H39" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I39" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -1925,24 +1926,24 @@
         <v>38</v>
       </c>
       <c r="F40" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G40">
         <v>8</v>
       </c>
       <c r="H40" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="I40" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="C41">
         <v>0</v>
@@ -1955,24 +1956,24 @@
         <v>65</v>
       </c>
       <c r="F41" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G41">
         <v>9</v>
       </c>
       <c r="H41" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I41" t="s">
-        <v>110</v>
+        <v>77</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>73</v>
+        <v>101</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="C42">
         <v>0</v>
@@ -1985,24 +1986,24 @@
         <v>44</v>
       </c>
       <c r="F42" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G42">
         <v>9</v>
       </c>
       <c r="H42" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I42" t="s">
-        <v>110</v>
+        <v>77</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>75</v>
+        <v>102</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -2015,24 +2016,24 @@
         <v>19</v>
       </c>
       <c r="F43" t="s">
-        <v>102</v>
+        <v>69</v>
       </c>
       <c r="G43">
         <v>4</v>
       </c>
       <c r="H43" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="I43" t="s">
-        <v>110</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>113</v>
+        <v>82</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="C44">
         <v>0</v>
@@ -2045,24 +2046,24 @@
         <v>32</v>
       </c>
       <c r="F44" t="s">
-        <v>106</v>
+        <v>73</v>
       </c>
       <c r="G44">
         <v>3</v>
       </c>
       <c r="H44" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I44" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>113</v>
+        <v>82</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="C45">
         <v>32</v>
@@ -2075,24 +2076,24 @@
         <v>28</v>
       </c>
       <c r="F45" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="G45">
         <v>6</v>
       </c>
       <c r="H45" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I45" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>89</v>
+        <v>58</v>
       </c>
       <c r="C46">
         <v>0</v>
@@ -2105,24 +2106,24 @@
         <v>87</v>
       </c>
       <c r="F46" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="G46">
         <v>6</v>
       </c>
       <c r="H46" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I46" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>80</v>
+        <v>52</v>
       </c>
       <c r="C47">
         <v>0</v>
@@ -2135,24 +2136,24 @@
         <v>30</v>
       </c>
       <c r="F47" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="G47">
         <v>1</v>
       </c>
       <c r="H47" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I47" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>81</v>
+        <v>53</v>
       </c>
       <c r="C48">
         <v>30</v>
@@ -2165,24 +2166,24 @@
         <v>20</v>
       </c>
       <c r="F48" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="G48">
         <v>6</v>
       </c>
       <c r="H48" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I48" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>83</v>
+        <v>54</v>
       </c>
       <c r="C49">
         <v>0</v>
@@ -2195,24 +2196,24 @@
         <v>20</v>
       </c>
       <c r="F49" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="G49">
         <v>1</v>
       </c>
       <c r="H49" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I49" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="C50">
         <v>20</v>
@@ -2225,24 +2226,24 @@
         <v>20</v>
       </c>
       <c r="F50" t="s">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="G50">
         <v>5</v>
       </c>
       <c r="H50" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I50" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>92</v>
+        <v>61</v>
       </c>
       <c r="C51">
         <v>40</v>
@@ -2255,24 +2256,24 @@
         <v>55</v>
       </c>
       <c r="F51" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G51">
         <v>8</v>
       </c>
       <c r="H51" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I51" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>84</v>
+        <v>106</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="C52">
         <v>0</v>
@@ -2285,24 +2286,24 @@
         <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>104</v>
+        <v>71</v>
       </c>
       <c r="G52">
         <v>1</v>
       </c>
       <c r="H52" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I52" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>84</v>
+        <v>106</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="C53">
         <v>10</v>
@@ -2315,24 +2316,24 @@
         <v>20</v>
       </c>
       <c r="F53" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="G53">
         <v>6</v>
       </c>
       <c r="H53" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I53" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>84</v>
+        <v>106</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>94</v>
+        <v>63</v>
       </c>
       <c r="C54">
         <v>30</v>
@@ -2345,24 +2346,24 @@
         <v>64</v>
       </c>
       <c r="F54" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G54">
         <v>8</v>
       </c>
       <c r="H54" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I54" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>95</v>
+        <v>64</v>
       </c>
       <c r="C55">
         <v>0</v>
@@ -2375,16 +2376,16 @@
         <v>63</v>
       </c>
       <c r="F55" t="s">
-        <v>105</v>
+        <v>72</v>
       </c>
       <c r="G55">
         <v>7</v>
       </c>
       <c r="H55" t="s">
-        <v>100</v>
+        <v>67</v>
       </c>
       <c r="I55" t="s">
-        <v>108</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>